<commit_message>
bug found in threshold failure of >2 continguous runs meeting threshold
</commit_message>
<xml_diff>
--- a/OUTPUT/LexA/Staph_LexA_Q9L4P1.xlsx
+++ b/OUTPUT/LexA/Staph_LexA_Q9L4P1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,27 +466,85 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[(8, 5), (9, 4), (10, 3), (11, 2), (12, 1)]</t>
+          <t>[(8, 5), (9, 4), (10, 3), (11, 2), (12, 1), (13, 0)]</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>7.930041115930132</v>
+        <v>11.99999993760844</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TGTTC</t>
+          <t>TGTACA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ACAAG</t>
+          <t>ACATGT</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>0.0046</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>[(3, 2), (4, 1), (5, 0)]</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5.999999968804222</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ACA</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0.6868</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>[(11, 10), (12, 9), (13, 8)]</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>5.999999968804222</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ACA</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>TGT</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0.6868</v>
       </c>
     </row>
   </sheetData>

</xml_diff>